<commit_message>
Balans: 2x zywnosc do wzrostu miasta (wszystkie warianty + poziomy trudnosci) + regen paneli
Maciej: podwoic prog zywnosci do rozwoju miasta. Prog = (10 + N x wsp) x mnoznik_trudnosci/tempa.
Mnozniki tylko MNOZA baze, wiec podwojenie bazy podwaja dla WSZYSTKICH trudnosci/temp:
- economy.ts:737 + turn-economy.ts:588: baza 10 -> 20 (oba miejsca liczace prog).
- econ-params.json prog_wzrostu_wspolczynnik: easy 6->12, normal 8->16, hard 10->20 (kazdy poziom).
=> prog = 20 + N x (2*wsp) = 2 x (10 + N x wsp), dokladny x2 wszedzie.

Panele sterowania: zregenerowane wszystkie 5 (gen-panel-a..e z gra/data). Panel-B (ekonomia) padal
na PRE-ISTNIEJACYM bugu (openpyxl nie zapisze listy [2,1,1,0] do komorki) -> dodany helper _cell()
konwertujacy listy/dicty na string; Panel-B regeneruje sie poprawnie.

tsc=0, smoke OK, JSON valid. Deploy 0ea5d61f.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/panele-sterowania/Panel-D.xlsx
+++ b/panele-sterowania/Panel-D.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -477,16 +477,19 @@
           <t>Panel sterowania — Grupa D (Cywilizacje, Dyplomacja, AI, Barbarzyńcy)</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Wygenerowano: 2026-07-04 22:11</t>
-        </is>
-      </c>
+          <t>Wygenerowano: 2026-07-09 18:14</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -494,6 +497,7 @@
           <t>JAK UŻYWAĆ</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -501,6 +505,7 @@
           <t>1. Edytuj kolumnę Wartość (parametry) lub komórki w arkuszach tabelarycznych.</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -508,6 +513,7 @@
           <t>2. Zapisz plik Panel-D.xlsx.</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -515,9 +521,11 @@
           <t>3. Napisz w czacie grupy D: eksportuj panel — agent odpali export-d.py.</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -525,6 +533,7 @@
           <t>Arkusze tabelaryczne: Bonusy-cywilizacji, Cywilizacje-roster, Parametry-cyw, AI-per-nacja, Dyplomacja-akcje, Dyplomacja-per-nacja.</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -532,56 +541,7 @@
           <t>Spec: docs/obieg/PANEL-STEROWANIA-SPEC.md</t>
         </is>
       </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>SYNC CYW 2026-07-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Zrodlo: gra/data/*.json (15 nacji, roster-6, archetypy Q7=A)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Hetyci: archetype_hetyci_nauka_priorytet = 2 (Maciej)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Babilonia: nauka +2, wojsko -1 (bez minusa na nauce)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Celtowie: Soldurii w bonusy (decyzja CELT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Eksport: CZEKA sygnalu Macieja po edycji Wartosc w Excelu</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Ostatni sync: 2026-07-04 22:11</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>